<commit_message>
Added RAD Test Suites
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/UM-Data.xlsx
+++ b/KatalonData/Bootstrap/UM-Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\Bootstrap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{6C31231A-6620-466E-B6BB-695AE682D6A1}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr documentId="13_ncr:1_{7B68E34D-93B4-40FB-B2DA-4965D8FF65C5}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView activeTab="6" firstSheet="3" windowHeight="15675" windowWidth="28996" xWindow="-98" xr2:uid="{354FC140-4496-4D7F-AB69-566E59F6C646}" yWindow="-98"/>
+    <workbookView activeTab="5" firstSheet="3" windowHeight="16776" windowWidth="30936" xWindow="45972" xr2:uid="{354FC140-4496-4D7F-AB69-566E59F6C646}" yWindow="2952"/>
   </bookViews>
   <sheets>
     <sheet name="CreateUser" r:id="rId1" sheetId="1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="292">
   <si>
     <t>Result</t>
   </si>
@@ -209,9 +209,6 @@
     <t>Username is not unique</t>
   </si>
   <si>
-    <t>Hello@2222</t>
-  </si>
-  <si>
     <t>OVK67648</t>
   </si>
   <si>
@@ -353,9 +350,6 @@
     <t>Hello@5555555</t>
   </si>
   <si>
-    <t>Thu Jun 29 09:15:41 EDT 2023</t>
-  </si>
-  <si>
     <t>Thu Jun 29 09:15:59 EDT 2023</t>
   </si>
   <si>
@@ -641,15 +635,6 @@
     <t>Sat Nov 15 18:30:05 EST 2025</t>
   </si>
   <si>
-    <t>Tue Feb 17 22:05:16 EST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 17 22:05:59 EST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 17 22:06:41 EST 2026</t>
-  </si>
-  <si>
     <t>Tue Feb 17 22:07:26 EST 2026</t>
   </si>
   <si>
@@ -866,37 +851,88 @@
     <t>Hello@1111111</t>
   </si>
   <si>
-    <t>Fri Feb 20 21:12:20 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:12:37 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:12:48 EST 2026</t>
+    <t>Fri Feb 20 21:15:10 EST 2026</t>
+  </si>
+  <si>
+    <t>Fri Feb 20 21:15:21 EST 2026</t>
+  </si>
+  <si>
+    <t>Fri Feb 20 21:15:30 EST 2026</t>
+  </si>
+  <si>
+    <t>Fri Feb 20 21:16:39 EST 2026</t>
+  </si>
+  <si>
+    <t>Fri Feb 20 21:16:50 EST 2026</t>
+  </si>
+  <si>
+    <t>Fri Feb 20 21:17:00 EST 2026</t>
+  </si>
+  <si>
+    <t>Mon Feb 23 11:43:52 EST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 18:06:22 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 18:07:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 18:07:56 EDT 2026</t>
+  </si>
+  <si>
+    <t>Hello@3333333</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Fri Feb 20 21:15:10 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:15:21 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:15:30 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:16:39 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:16:50 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:17:00 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 23 11:43:52 EST 2026</t>
+    <t>Thu Jun 04 16:14:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:15:48 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:16:36 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:17:23 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:31:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:32:12 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:32:29 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:32:46 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:33:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:33:27 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:33:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:33:59 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:34:16 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:34:32 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:34:48 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu Jun 04 16:35:04 EDT 2026</t>
   </si>
 </sst>
 </file>
@@ -963,7 +999,7 @@
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
     <xf applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="2" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
     <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
       <alignment wrapText="1"/>
@@ -974,6 +1010,7 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="1"/>
     <xf applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0"/>
+    <xf applyFill="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle builtinId="8" name="Hyperlink" xfId="1"/>
@@ -1343,10 +1380,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>194</v>
+        <v>271</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -1358,10 +1395,10 @@
         <v>13</v>
       </c>
       <c r="I2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>14</v>
@@ -1369,10 +1406,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>195</v>
+        <v>272</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -1384,10 +1421,10 @@
         <v>13</v>
       </c>
       <c r="I3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>14</v>
@@ -1395,10 +1432,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>196</v>
+        <v>273</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -1410,10 +1447,10 @@
         <v>13</v>
       </c>
       <c r="I4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>14</v>
@@ -1472,16 +1509,16 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>256</v>
+        <v>280</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>27</v>
@@ -1489,10 +1526,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>281</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -1506,16 +1543,16 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>252</v>
+        <v>282</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>29</v>
@@ -1523,10 +1560,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>243</v>
+        <v>283</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -1540,10 +1577,10 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>244</v>
+        <v>284</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
@@ -1557,10 +1594,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>245</v>
+        <v>285</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
@@ -1574,10 +1611,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>246</v>
+        <v>286</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
@@ -1591,10 +1628,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>247</v>
+        <v>287</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
@@ -1608,10 +1645,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>248</v>
+        <v>288</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>11</v>
@@ -1625,10 +1662,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>249</v>
+        <v>289</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>11</v>
@@ -1642,10 +1679,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>250</v>
+        <v>290</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
@@ -1659,10 +1696,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>251</v>
+        <v>291</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>11</v>
@@ -1726,17 +1763,17 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1746,10 +1783,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
@@ -1770,7 +1807,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1969,10 +2006,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -1990,10 +2027,10 @@
         <v>41</v>
       </c>
       <c r="I2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>14</v>
@@ -2004,10 +2041,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -2025,10 +2062,10 @@
         <v>42</v>
       </c>
       <c r="I3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>14</v>
@@ -2039,10 +2076,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -2060,10 +2097,10 @@
         <v>13</v>
       </c>
       <c r="I4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>14</v>
@@ -2074,10 +2111,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -2095,10 +2132,10 @@
         <v>13</v>
       </c>
       <c r="I5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>14</v>
@@ -2109,16 +2146,16 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>46</v>
@@ -2130,30 +2167,30 @@
         <v>13</v>
       </c>
       <c r="I6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row ht="28.5" r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>46</v>
@@ -2165,30 +2202,30 @@
         <v>13</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="J7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>46</v>
@@ -2200,30 +2237,30 @@
         <v>13</v>
       </c>
       <c r="I8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>46</v>
@@ -2235,30 +2272,30 @@
         <v>13</v>
       </c>
       <c r="I9" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>46</v>
@@ -2270,30 +2307,30 @@
         <v>13</v>
       </c>
       <c r="I10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>46</v>
@@ -2305,30 +2342,30 @@
         <v>13</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>46</v>
@@ -2340,33 +2377,33 @@
         <v>13</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row ht="28.5" r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F13" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>47</v>
@@ -2375,51 +2412,51 @@
         <v>13</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row ht="28.5" r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B14" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F14" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G14" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="I14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="J14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.45">
@@ -2484,682 +2521,682 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" t="s">
         <v>51</v>
-      </c>
-      <c r="F2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
         <v>51</v>
-      </c>
-      <c r="F4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" t="s">
         <v>51</v>
-      </c>
-      <c r="F6" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" t="s">
         <v>51</v>
-      </c>
-      <c r="F8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" t="s">
         <v>51</v>
-      </c>
-      <c r="F10" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F12" t="s">
         <v>51</v>
-      </c>
-      <c r="F12" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" t="s">
         <v>51</v>
-      </c>
-      <c r="F14" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" t="s">
         <v>51</v>
-      </c>
-      <c r="F16" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" t="s">
         <v>51</v>
-      </c>
-      <c r="F18" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F20" t="s">
         <v>51</v>
-      </c>
-      <c r="F20" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" t="s">
         <v>51</v>
-      </c>
-      <c r="F22" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" t="s">
         <v>51</v>
-      </c>
-      <c r="F24" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F26" t="s">
         <v>51</v>
-      </c>
-      <c r="F26" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B27" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" t="s">
         <v>51</v>
-      </c>
-      <c r="F28" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F30" t="s">
         <v>51</v>
-      </c>
-      <c r="F30" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F31" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" t="s">
         <v>51</v>
-      </c>
-      <c r="F32" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B34" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E34" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F34" t="s">
         <v>51</v>
-      </c>
-      <c r="F34" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B35" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F36" t="s">
         <v>51</v>
-      </c>
-      <c r="F36" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" t="s">
         <v>51</v>
-      </c>
-      <c r="F38" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B39" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B40" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F40" t="s">
         <v>51</v>
-      </c>
-      <c r="F40" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B41" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F41" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -3196,10 +3233,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -3207,10 +3244,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
@@ -3218,10 +3255,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -3229,10 +3266,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -3240,10 +3277,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -3251,10 +3288,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -3262,10 +3299,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -3273,10 +3310,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -3284,10 +3321,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -3295,10 +3332,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -3306,10 +3343,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -3317,10 +3354,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -3328,10 +3365,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -3339,10 +3376,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -3350,10 +3387,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -3361,10 +3398,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B17" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -3372,10 +3409,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -3383,10 +3420,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -3394,10 +3431,10 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
@@ -3405,10 +3442,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
@@ -3416,10 +3453,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
@@ -3427,10 +3464,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B23" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
@@ -3438,10 +3475,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
@@ -3449,10 +3486,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
@@ -3460,10 +3497,10 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
@@ -3471,10 +3508,10 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B27" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
@@ -3482,10 +3519,10 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
@@ -3493,10 +3530,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
@@ -3504,10 +3541,10 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
@@ -3515,10 +3552,10 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
@@ -3568,10 +3605,10 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>5</v>
@@ -3594,19 +3631,19 @@
     </row>
     <row ht="28.5" r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G2" s="3">
         <v>9</v>
@@ -3615,19 +3652,19 @@
     </row>
     <row ht="28.5" r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="G3" s="3">
         <v>9</v>
@@ -3636,19 +3673,19 @@
     </row>
     <row ht="28.5" r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G4" s="3">
         <v>9</v>
@@ -3656,19 +3693,19 @@
     </row>
     <row ht="28.5" r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G5" s="3">
         <v>9</v>
@@ -3676,19 +3713,19 @@
     </row>
     <row ht="28.5" r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G6" s="3">
         <v>9</v>
@@ -3696,19 +3733,19 @@
     </row>
     <row ht="28.5" r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G7" s="3">
         <v>9</v>
@@ -3716,19 +3753,19 @@
     </row>
     <row ht="28.5" r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G8" s="3">
         <v>9</v>
@@ -3736,19 +3773,19 @@
     </row>
     <row ht="28.5" r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G9" s="3">
         <v>9</v>
@@ -3756,19 +3793,19 @@
     </row>
     <row ht="28.5" r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G10" s="3">
         <v>10</v>
@@ -3776,19 +3813,19 @@
     </row>
     <row ht="28.5" r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G11" s="3">
         <v>10</v>
@@ -3796,19 +3833,19 @@
     </row>
     <row ht="28.5" r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G12" s="3">
         <v>10</v>
@@ -3816,19 +3853,19 @@
     </row>
     <row ht="28.5" r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G13" s="3">
         <v>10</v>
@@ -3836,19 +3873,19 @@
     </row>
     <row ht="28.5" r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G14" s="3">
         <v>10</v>
@@ -3856,19 +3893,19 @@
     </row>
     <row ht="28.5" r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G15" s="3">
         <v>10</v>
@@ -3876,19 +3913,19 @@
     </row>
     <row ht="28.5" r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G16" s="3">
         <v>10</v>
@@ -3896,19 +3933,19 @@
     </row>
     <row ht="28.5" r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G17" s="3">
         <v>10</v>
@@ -3977,10 +4014,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -3992,10 +4029,10 @@
         <v>13</v>
       </c>
       <c r="I2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>14</v>
@@ -4003,10 +4040,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4018,10 +4055,10 @@
         <v>13</v>
       </c>
       <c r="I3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>14</v>
@@ -4074,33 +4111,33 @@
         <v>26</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>27</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J2" s="3">
         <v>9</v>
@@ -4108,22 +4145,22 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>27</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J3" s="3">
         <v>9</v>
@@ -4136,13 +4173,13 @@
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>27</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J4" s="3">
         <v>9</v>
@@ -4155,13 +4192,13 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>27</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J5" s="3">
         <v>9</v>
@@ -4174,13 +4211,13 @@
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>27</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J6" s="3">
         <v>9</v>
@@ -4190,19 +4227,19 @@
       <c r="A7"/>
       <c r="B7"/>
       <c r="C7" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>27</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J7" s="3">
         <v>9</v>
@@ -4215,13 +4252,13 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>27</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J8" s="3">
         <v>9</v>
@@ -4275,27 +4312,27 @@
         <v>26</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -4303,7 +4340,7 @@
         <v>27</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J2" s="3">
         <v>9</v>
@@ -4311,17 +4348,17 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -4329,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J3" s="3">
         <v>9</v>
@@ -4341,7 +4378,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -4349,7 +4386,7 @@
         <v>27</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J4" s="3">
         <v>9</v>
@@ -4361,7 +4398,7 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -4369,7 +4406,7 @@
         <v>27</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J5" s="3">
         <v>9</v>
@@ -4381,7 +4418,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -4389,7 +4426,7 @@
         <v>27</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J6" s="3">
         <v>9</v>
@@ -4397,13 +4434,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="C7" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -4411,7 +4448,7 @@
         <v>27</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J7" s="3">
         <v>9</v>
@@ -4423,7 +4460,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -4431,7 +4468,7 @@
         <v>27</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J8" s="3">
         <v>9</v>
@@ -4469,7 +4506,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>26</v>
@@ -4477,16 +4514,16 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>186</v>
+        <v>276</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>27</v>
@@ -4494,16 +4531,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>187</v>
+        <v>277</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>27</v>
@@ -4511,16 +4548,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>188</v>
+        <v>278</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>27</v>
@@ -4528,16 +4565,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>189</v>
+        <v>279</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>27</v>
@@ -4608,10 +4645,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -4626,10 +4663,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4644,10 +4681,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -4662,10 +4699,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -4680,10 +4717,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
@@ -4698,10 +4735,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
@@ -4749,7 +4786,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>26</v>
@@ -4757,16 +4794,16 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>27</v>
@@ -4774,16 +4811,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>28</v>
@@ -4791,16 +4828,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>29</v>
@@ -4808,16 +4845,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>30</v>
@@ -4859,10 +4896,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -4873,10 +4910,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4887,10 +4924,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -4901,10 +4938,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -4949,10 +4986,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -4963,10 +5000,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4977,10 +5014,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -4991,10 +5028,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -5072,10 +5109,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -5090,10 +5127,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -5108,10 +5145,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -5167,10 +5204,10 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -5178,16 +5215,16 @@
       <c r="E2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F2" t="s">
-        <v>50</v>
+      <c r="F2" s="6" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -5195,16 +5232,16 @@
       <c r="E3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F3" t="s">
-        <v>50</v>
+      <c r="F3" s="6" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -5212,8 +5249,8 @@
       <c r="E4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F4" t="s">
-        <v>50</v>
+      <c r="F4" s="6" t="s">
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -5260,56 +5297,56 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>263</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -5358,10 +5395,10 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -5370,7 +5407,7 @@
         <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -5413,20 +5450,20 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>